<commit_message>
In Config file, change Process Group List to reflect LIB processes; in Classifications file, change Eng. Mats and End Use sectors tabs to better match LIB materials
</commit_message>
<xml_diff>
--- a/docs/Files/ODYM_Classifications_EV_LIB.xlsx
+++ b/docs/Files/ODYM_Classifications_EV_LIB.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FAE011-8F8D-4A76-ACBF-2C8D0ED6DAE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6250B6-954C-46E6-9662-719CED7DC4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="749" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="749" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover_Dimensions_Aspects" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="283">
   <si>
     <t>Name</t>
   </si>
@@ -848,18 +848,6 @@
     <t>d70ff49d-88c3-4a52-a12e-14ec6f53984f</t>
   </si>
   <si>
-    <t>construction</t>
-  </si>
-  <si>
-    <t>products and other</t>
-  </si>
-  <si>
-    <t>vehicles</t>
-  </si>
-  <si>
-    <t>machinery</t>
-  </si>
-  <si>
     <t>Scenario</t>
   </si>
   <si>
@@ -891,6 +879,12 @@
   </si>
   <si>
     <t>LIB scrap</t>
+  </si>
+  <si>
+    <t>EV LIB</t>
+  </si>
+  <si>
+    <t>other LIB products</t>
   </si>
 </sst>
 </file>
@@ -1293,7 +1287,7 @@
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -1301,7 +1295,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -1309,7 +1303,7 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -1828,7 +1822,7 @@
       </c>
       <c r="F11" t="str">
         <f>End_Use_Sectors!D2</f>
-        <v>vehicles</v>
+        <v>EV LIB</v>
       </c>
       <c r="G11" t="str">
         <f>Waste_Scrap!D2</f>
@@ -1859,9 +1853,9 @@
         <f>Engineering_Materials!D3</f>
         <v>Automotive steel</v>
       </c>
-      <c r="F12" t="str">
-        <f>End_Use_Sectors!D3</f>
-        <v>machinery</v>
+      <c r="F12" t="e">
+        <f>End_Use_Sectors!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="G12" t="str">
         <f>Waste_Scrap!D3</f>
@@ -1888,9 +1882,9 @@
         <f>Chemical_Elements!D4</f>
         <v>He</v>
       </c>
-      <c r="F13" t="str">
+      <c r="F13">
         <f>End_Use_Sectors!D4</f>
-        <v>construction</v>
+        <v>0</v>
       </c>
       <c r="H13" t="str">
         <f>'10_Regions'!D4</f>
@@ -1910,8 +1904,8 @@
         <v>Li</v>
       </c>
       <c r="F14" t="str">
-        <f>End_Use_Sectors!D5</f>
-        <v>products and other</v>
+        <f>End_Use_Sectors!D3</f>
+        <v>other LIB products</v>
       </c>
       <c r="H14" t="str">
         <f>'10_Regions'!D5</f>
@@ -25737,7 +25731,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26272,7 +26266,7 @@
         <v>224</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26459,7 +26453,7 @@
         <v>224</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26473,8 +26467,8 @@
       <c r="B3" t="s">
         <v>240</v>
       </c>
-      <c r="D3" t="s">
-        <v>273</v>
+      <c r="D3" s="1" t="s">
+        <v>282</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26488,12 +26482,7 @@
       <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
+      <c r="D4" s="1"/>
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -26502,12 +26491,6 @@
       </c>
       <c r="B5" t="s">
         <v>268</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="E5">
-        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -26655,7 +26638,7 @@
         <v>224</v>
       </c>
       <c r="D2" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26838,7 +26821,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26855,10 +26838,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="D2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26871,10 +26854,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="D3" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26897,7 +26880,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>

</xml_diff>

<commit_message>
Changed descriptions for End use sectors and waste scrap tabs in classifications file
</commit_message>
<xml_diff>
--- a/docs/Files/ODYM_Classifications_EV_LIB.xlsx
+++ b/docs/Files/ODYM_Classifications_EV_LIB.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F3D0BA-1ABD-4913-A82D-37810B77147D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB61B992-619F-41A2-B403-DA0DA53277C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="749" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="749" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover_Dimensions_Aspects" sheetId="8" r:id="rId1"/>
@@ -779,9 +779,6 @@
     <t>Lists of engineering materials (in the narrower sense), output of engineering material production industries.</t>
   </si>
   <si>
-    <t>Steel shred</t>
-  </si>
-  <si>
     <t>ODYM Classifications master file, tutorial version</t>
   </si>
   <si>
@@ -881,10 +878,13 @@
     <t>EV LIB</t>
   </si>
   <si>
-    <t>other LIB products</t>
-  </si>
-  <si>
     <t>LIB materials</t>
+  </si>
+  <si>
+    <t>other EV LIB products</t>
+  </si>
+  <si>
+    <t>Other scrap</t>
   </si>
 </sst>
 </file>
@@ -1282,12 +1282,12 @@
   <sheetData>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -1295,7 +1295,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -1303,7 +1303,7 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -1855,11 +1855,11 @@
       </c>
       <c r="F12" t="str">
         <f>End_Use_Sectors!D3</f>
-        <v>other LIB products</v>
+        <v>other EV LIB products</v>
       </c>
       <c r="G12" t="str">
         <f>Waste_Scrap!D3</f>
-        <v>Steel shred</v>
+        <v>Other scrap</v>
       </c>
       <c r="H12" t="str">
         <f>'10_Regions'!D3</f>
@@ -25675,7 +25675,7 @@
     </row>
     <row r="103" spans="4:6" x14ac:dyDescent="0.3">
       <c r="D103" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E103">
         <v>101</v>
@@ -25702,7 +25702,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -25723,7 +25723,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -25735,10 +25735,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -25753,7 +25753,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -25765,10 +25765,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -25783,7 +25783,7 @@
         <v>43487</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -25798,7 +25798,7 @@
         <v>43487</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E7">
         <v>5</v>
@@ -25813,7 +25813,7 @@
         <v>15</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E8">
         <v>6</v>
@@ -25826,7 +25826,7 @@
       </c>
       <c r="B9" s="3"/>
       <c r="D9" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E9">
         <v>7</v>
@@ -25835,7 +25835,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D10" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E10">
         <v>8</v>
@@ -25844,7 +25844,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D11" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E11">
         <v>9</v>
@@ -25853,7 +25853,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D12" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E12">
         <v>10</v>
@@ -26238,7 +26238,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26258,7 +26258,7 @@
         <v>224</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26273,7 +26273,7 @@
         <v>246</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26295,7 +26295,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D5" s="1"/>
       <c r="F5" s="1"/>
@@ -26424,7 +26424,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26445,7 +26445,7 @@
         <v>224</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26482,7 +26482,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -26610,7 +26610,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26630,7 +26630,7 @@
         <v>224</v>
       </c>
       <c r="D2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26647,7 +26647,7 @@
         <v>240</v>
       </c>
       <c r="D3" t="s">
-        <v>247</v>
+        <v>282</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26671,7 +26671,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>
@@ -26813,7 +26813,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>10</v>
@@ -26830,10 +26830,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -26846,10 +26846,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -26872,7 +26872,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" s="1"/>

</xml_diff>